<commit_message>
Lower the one room starting price to £1,650
The single room price, a 2.0 or 2.5kW wall mounted split, drops from
£1,850 to £1,650 to compete with local installers. Other sizes, multi
splits and commercial prices are unchanged.

Changed everywhere it appears, 66 places: page copy, meta and social
descriptions, the price list, the hero stats, the HVACBusiness and
Service structured data (minPrice, price), the calculator in main.js,
the town page generator, the four guides, llms.txt key facts, the CMS
config comment, the README, and the Excel and CSV sizing tools, with
the workbook regenerated. Generated pages rebuilt from source. No
£1,850 remains anywhere in the repo; the calculator now returns
"from £1,650 fitted" for a small room.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tools/coolin-sizing.xlsx
+++ b/tools/coolin-sizing.xlsx
@@ -268,7 +268,7 @@
         </is>
       </c>
       <c r="B14" s="6">
-        <f>IF(B12&lt;=2.0,1850,IF(B12&lt;=2.5,1850,IF(B12&lt;=3.5,1995,IF(B12&lt;=5.0,2280,IF(B12&lt;=6.0,2650,IF(B12&lt;=7.1,2950,""))))))</f>
+        <f>IF(B12&lt;=2.0,1650,IF(B12&lt;=2.5,1650,IF(B12&lt;=3.5,1995,IF(B12&lt;=5.0,2280,IF(B12&lt;=6.0,2650,IF(B12&lt;=7.1,2950,""))))))</f>
       </c>
       <c r="C14" s="5" t="inlineStr">
         <is>
@@ -402,7 +402,7 @@
         <f>IF(J18="","",IF(J18&lt;=2.0,2.0,IF(J18&lt;=2.5,2.5,IF(J18&lt;=3.5,3.5,IF(J18&lt;=5.0,5.0,IF(J18&lt;=6.0,6.0,IF(J18&lt;=7.1,7.1,"two units")))))))</f>
       </c>
       <c r="L18" s="6">
-        <f>IF(J18="","",IF(J18&lt;=2.0,1850,IF(J18&lt;=2.5,1850,IF(J18&lt;=3.5,1995,IF(J18&lt;=5.0,2280,IF(J18&lt;=6.0,2650,IF(J18&lt;=7.1,2950,"")))))))</f>
+        <f>IF(J18="","",IF(J18&lt;=2.0,1650,IF(J18&lt;=2.5,1650,IF(J18&lt;=3.5,1995,IF(J18&lt;=5.0,2280,IF(J18&lt;=6.0,2650,IF(J18&lt;=7.1,2950,"")))))))</f>
       </c>
     </row>
     <row r="19">
@@ -450,7 +450,7 @@
         <f>IF(J19="","",IF(J19&lt;=2.0,2.0,IF(J19&lt;=2.5,2.5,IF(J19&lt;=3.5,3.5,IF(J19&lt;=5.0,5.0,IF(J19&lt;=6.0,6.0,IF(J19&lt;=7.1,7.1,"two units")))))))</f>
       </c>
       <c r="L19" s="6">
-        <f>IF(J19="","",IF(J19&lt;=2.0,1850,IF(J19&lt;=2.5,1850,IF(J19&lt;=3.5,1995,IF(J19&lt;=5.0,2280,IF(J19&lt;=6.0,2650,IF(J19&lt;=7.1,2950,"")))))))</f>
+        <f>IF(J19="","",IF(J19&lt;=2.0,1650,IF(J19&lt;=2.5,1650,IF(J19&lt;=3.5,1995,IF(J19&lt;=5.0,2280,IF(J19&lt;=6.0,2650,IF(J19&lt;=7.1,2950,"")))))))</f>
       </c>
     </row>
     <row r="20">
@@ -498,7 +498,7 @@
         <f>IF(J20="","",IF(J20&lt;=2.0,2.0,IF(J20&lt;=2.5,2.5,IF(J20&lt;=3.5,3.5,IF(J20&lt;=5.0,5.0,IF(J20&lt;=6.0,6.0,IF(J20&lt;=7.1,7.1,"two units")))))))</f>
       </c>
       <c r="L20" s="6">
-        <f>IF(J20="","",IF(J20&lt;=2.0,1850,IF(J20&lt;=2.5,1850,IF(J20&lt;=3.5,1995,IF(J20&lt;=5.0,2280,IF(J20&lt;=6.0,2650,IF(J20&lt;=7.1,2950,"")))))))</f>
+        <f>IF(J20="","",IF(J20&lt;=2.0,1650,IF(J20&lt;=2.5,1650,IF(J20&lt;=3.5,1995,IF(J20&lt;=5.0,2280,IF(J20&lt;=6.0,2650,IF(J20&lt;=7.1,2950,"")))))))</f>
       </c>
     </row>
     <row r="21">
@@ -520,7 +520,7 @@
         <f>IF(J21="","",IF(J21&lt;=2.0,2.0,IF(J21&lt;=2.5,2.5,IF(J21&lt;=3.5,3.5,IF(J21&lt;=5.0,5.0,IF(J21&lt;=6.0,6.0,IF(J21&lt;=7.1,7.1,"two units")))))))</f>
       </c>
       <c r="L21" s="6">
-        <f>IF(J21="","",IF(J21&lt;=2.0,1850,IF(J21&lt;=2.5,1850,IF(J21&lt;=3.5,1995,IF(J21&lt;=5.0,2280,IF(J21&lt;=6.0,2650,IF(J21&lt;=7.1,2950,"")))))))</f>
+        <f>IF(J21="","",IF(J21&lt;=2.0,1650,IF(J21&lt;=2.5,1650,IF(J21&lt;=3.5,1995,IF(J21&lt;=5.0,2280,IF(J21&lt;=6.0,2650,IF(J21&lt;=7.1,2950,"")))))))</f>
       </c>
     </row>
     <row r="22">
@@ -542,7 +542,7 @@
         <f>IF(J22="","",IF(J22&lt;=2.0,2.0,IF(J22&lt;=2.5,2.5,IF(J22&lt;=3.5,3.5,IF(J22&lt;=5.0,5.0,IF(J22&lt;=6.0,6.0,IF(J22&lt;=7.1,7.1,"two units")))))))</f>
       </c>
       <c r="L22" s="6">
-        <f>IF(J22="","",IF(J22&lt;=2.0,1850,IF(J22&lt;=2.5,1850,IF(J22&lt;=3.5,1995,IF(J22&lt;=5.0,2280,IF(J22&lt;=6.0,2650,IF(J22&lt;=7.1,2950,"")))))))</f>
+        <f>IF(J22="","",IF(J22&lt;=2.0,1650,IF(J22&lt;=2.5,1650,IF(J22&lt;=3.5,1995,IF(J22&lt;=5.0,2280,IF(J22&lt;=6.0,2650,IF(J22&lt;=7.1,2950,"")))))))</f>
       </c>
     </row>
     <row r="23">
@@ -564,7 +564,7 @@
         <f>IF(J23="","",IF(J23&lt;=2.0,2.0,IF(J23&lt;=2.5,2.5,IF(J23&lt;=3.5,3.5,IF(J23&lt;=5.0,5.0,IF(J23&lt;=6.0,6.0,IF(J23&lt;=7.1,7.1,"two units")))))))</f>
       </c>
       <c r="L23" s="6">
-        <f>IF(J23="","",IF(J23&lt;=2.0,1850,IF(J23&lt;=2.5,1850,IF(J23&lt;=3.5,1995,IF(J23&lt;=5.0,2280,IF(J23&lt;=6.0,2650,IF(J23&lt;=7.1,2950,"")))))))</f>
+        <f>IF(J23="","",IF(J23&lt;=2.0,1650,IF(J23&lt;=2.5,1650,IF(J23&lt;=3.5,1995,IF(J23&lt;=5.0,2280,IF(J23&lt;=6.0,2650,IF(J23&lt;=7.1,2950,"")))))))</f>
       </c>
     </row>
     <row r="24">
@@ -586,7 +586,7 @@
         <f>IF(J24="","",IF(J24&lt;=2.0,2.0,IF(J24&lt;=2.5,2.5,IF(J24&lt;=3.5,3.5,IF(J24&lt;=5.0,5.0,IF(J24&lt;=6.0,6.0,IF(J24&lt;=7.1,7.1,"two units")))))))</f>
       </c>
       <c r="L24" s="6">
-        <f>IF(J24="","",IF(J24&lt;=2.0,1850,IF(J24&lt;=2.5,1850,IF(J24&lt;=3.5,1995,IF(J24&lt;=5.0,2280,IF(J24&lt;=6.0,2650,IF(J24&lt;=7.1,2950,"")))))))</f>
+        <f>IF(J24="","",IF(J24&lt;=2.0,1650,IF(J24&lt;=2.5,1650,IF(J24&lt;=3.5,1995,IF(J24&lt;=5.0,2280,IF(J24&lt;=6.0,2650,IF(J24&lt;=7.1,2950,"")))))))</f>
       </c>
     </row>
     <row r="25">
@@ -608,7 +608,7 @@
         <f>IF(J25="","",IF(J25&lt;=2.0,2.0,IF(J25&lt;=2.5,2.5,IF(J25&lt;=3.5,3.5,IF(J25&lt;=5.0,5.0,IF(J25&lt;=6.0,6.0,IF(J25&lt;=7.1,7.1,"two units")))))))</f>
       </c>
       <c r="L25" s="6">
-        <f>IF(J25="","",IF(J25&lt;=2.0,1850,IF(J25&lt;=2.5,1850,IF(J25&lt;=3.5,1995,IF(J25&lt;=5.0,2280,IF(J25&lt;=6.0,2650,IF(J25&lt;=7.1,2950,"")))))))</f>
+        <f>IF(J25="","",IF(J25&lt;=2.0,1650,IF(J25&lt;=2.5,1650,IF(J25&lt;=3.5,1995,IF(J25&lt;=5.0,2280,IF(J25&lt;=6.0,2650,IF(J25&lt;=7.1,2950,"")))))))</f>
       </c>
     </row>
     <row r="26">
@@ -630,7 +630,7 @@
         <f>IF(J26="","",IF(J26&lt;=2.0,2.0,IF(J26&lt;=2.5,2.5,IF(J26&lt;=3.5,3.5,IF(J26&lt;=5.0,5.0,IF(J26&lt;=6.0,6.0,IF(J26&lt;=7.1,7.1,"two units")))))))</f>
       </c>
       <c r="L26" s="6">
-        <f>IF(J26="","",IF(J26&lt;=2.0,1850,IF(J26&lt;=2.5,1850,IF(J26&lt;=3.5,1995,IF(J26&lt;=5.0,2280,IF(J26&lt;=6.0,2650,IF(J26&lt;=7.1,2950,"")))))))</f>
+        <f>IF(J26="","",IF(J26&lt;=2.0,1650,IF(J26&lt;=2.5,1650,IF(J26&lt;=3.5,1995,IF(J26&lt;=5.0,2280,IF(J26&lt;=6.0,2650,IF(J26&lt;=7.1,2950,"")))))))</f>
       </c>
     </row>
     <row r="27">
@@ -652,7 +652,7 @@
         <f>IF(J27="","",IF(J27&lt;=2.0,2.0,IF(J27&lt;=2.5,2.5,IF(J27&lt;=3.5,3.5,IF(J27&lt;=5.0,5.0,IF(J27&lt;=6.0,6.0,IF(J27&lt;=7.1,7.1,"two units")))))))</f>
       </c>
       <c r="L27" s="6">
-        <f>IF(J27="","",IF(J27&lt;=2.0,1850,IF(J27&lt;=2.5,1850,IF(J27&lt;=3.5,1995,IF(J27&lt;=5.0,2280,IF(J27&lt;=6.0,2650,IF(J27&lt;=7.1,2950,"")))))))</f>
+        <f>IF(J27="","",IF(J27&lt;=2.0,1650,IF(J27&lt;=2.5,1650,IF(J27&lt;=3.5,1995,IF(J27&lt;=5.0,2280,IF(J27&lt;=6.0,2650,IF(J27&lt;=7.1,2950,"")))))))</f>
       </c>
     </row>
     <row r="28">
@@ -674,7 +674,7 @@
         <f>IF(J28="","",IF(J28&lt;=2.0,2.0,IF(J28&lt;=2.5,2.5,IF(J28&lt;=3.5,3.5,IF(J28&lt;=5.0,5.0,IF(J28&lt;=6.0,6.0,IF(J28&lt;=7.1,7.1,"two units")))))))</f>
       </c>
       <c r="L28" s="6">
-        <f>IF(J28="","",IF(J28&lt;=2.0,1850,IF(J28&lt;=2.5,1850,IF(J28&lt;=3.5,1995,IF(J28&lt;=5.0,2280,IF(J28&lt;=6.0,2650,IF(J28&lt;=7.1,2950,"")))))))</f>
+        <f>IF(J28="","",IF(J28&lt;=2.0,1650,IF(J28&lt;=2.5,1650,IF(J28&lt;=3.5,1995,IF(J28&lt;=5.0,2280,IF(J28&lt;=6.0,2650,IF(J28&lt;=7.1,2950,"")))))))</f>
       </c>
     </row>
     <row r="29">
@@ -696,7 +696,7 @@
         <f>IF(J29="","",IF(J29&lt;=2.0,2.0,IF(J29&lt;=2.5,2.5,IF(J29&lt;=3.5,3.5,IF(J29&lt;=5.0,5.0,IF(J29&lt;=6.0,6.0,IF(J29&lt;=7.1,7.1,"two units")))))))</f>
       </c>
       <c r="L29" s="6">
-        <f>IF(J29="","",IF(J29&lt;=2.0,1850,IF(J29&lt;=2.5,1850,IF(J29&lt;=3.5,1995,IF(J29&lt;=5.0,2280,IF(J29&lt;=6.0,2650,IF(J29&lt;=7.1,2950,"")))))))</f>
+        <f>IF(J29="","",IF(J29&lt;=2.0,1650,IF(J29&lt;=2.5,1650,IF(J29&lt;=3.5,1995,IF(J29&lt;=5.0,2280,IF(J29&lt;=6.0,2650,IF(J29&lt;=7.1,2950,"")))))))</f>
       </c>
     </row>
     <row r="30">

</xml_diff>

<commit_message>
Even out the single room price ladder
After the starting price dropped to £1,650, the steps between sizes ran
+£345, +£285, +£370, +£300. Now round figures with an even climb:

  2.0 and 2.5 kW  £1,650
  3.5 kW          £1,850   (was £1,995)
  5.0 kW          £2,150   (was £2,280)
  6.0 kW          £2,450   (was £2,650, calculator only)
  7.1 kW          £2,750   (was £2,950)

Changed in the domestic price list, the cost guide's one room table,
the calculator, and the Excel and CSV sizing tools, with the workbook
rebuilt. Checked in the calculator: each size returns its new price.

Commercial prices are deliberately unchanged, including the 5kW wall
unit at £2,280 for a shop or office, since commercial work carries VAT
and more access and out of hours work.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tools/coolin-sizing.xlsx
+++ b/tools/coolin-sizing.xlsx
@@ -268,7 +268,7 @@
         </is>
       </c>
       <c r="B14" s="6">
-        <f>IF(B12&lt;=2.0,1650,IF(B12&lt;=2.5,1650,IF(B12&lt;=3.5,1995,IF(B12&lt;=5.0,2280,IF(B12&lt;=6.0,2650,IF(B12&lt;=7.1,2950,""))))))</f>
+        <f>IF(B12&lt;=2.0,1650,IF(B12&lt;=2.5,1650,IF(B12&lt;=3.5,1850,IF(B12&lt;=5.0,2150,IF(B12&lt;=6.0,2450,IF(B12&lt;=7.1,2750,""))))))</f>
       </c>
       <c r="C14" s="5" t="inlineStr">
         <is>
@@ -402,7 +402,7 @@
         <f>IF(J18="","",IF(J18&lt;=2.0,2.0,IF(J18&lt;=2.5,2.5,IF(J18&lt;=3.5,3.5,IF(J18&lt;=5.0,5.0,IF(J18&lt;=6.0,6.0,IF(J18&lt;=7.1,7.1,"two units")))))))</f>
       </c>
       <c r="L18" s="6">
-        <f>IF(J18="","",IF(J18&lt;=2.0,1650,IF(J18&lt;=2.5,1650,IF(J18&lt;=3.5,1995,IF(J18&lt;=5.0,2280,IF(J18&lt;=6.0,2650,IF(J18&lt;=7.1,2950,"")))))))</f>
+        <f>IF(J18="","",IF(J18&lt;=2.0,1650,IF(J18&lt;=2.5,1650,IF(J18&lt;=3.5,1850,IF(J18&lt;=5.0,2150,IF(J18&lt;=6.0,2450,IF(J18&lt;=7.1,2750,"")))))))</f>
       </c>
     </row>
     <row r="19">
@@ -450,7 +450,7 @@
         <f>IF(J19="","",IF(J19&lt;=2.0,2.0,IF(J19&lt;=2.5,2.5,IF(J19&lt;=3.5,3.5,IF(J19&lt;=5.0,5.0,IF(J19&lt;=6.0,6.0,IF(J19&lt;=7.1,7.1,"two units")))))))</f>
       </c>
       <c r="L19" s="6">
-        <f>IF(J19="","",IF(J19&lt;=2.0,1650,IF(J19&lt;=2.5,1650,IF(J19&lt;=3.5,1995,IF(J19&lt;=5.0,2280,IF(J19&lt;=6.0,2650,IF(J19&lt;=7.1,2950,"")))))))</f>
+        <f>IF(J19="","",IF(J19&lt;=2.0,1650,IF(J19&lt;=2.5,1650,IF(J19&lt;=3.5,1850,IF(J19&lt;=5.0,2150,IF(J19&lt;=6.0,2450,IF(J19&lt;=7.1,2750,"")))))))</f>
       </c>
     </row>
     <row r="20">
@@ -498,7 +498,7 @@
         <f>IF(J20="","",IF(J20&lt;=2.0,2.0,IF(J20&lt;=2.5,2.5,IF(J20&lt;=3.5,3.5,IF(J20&lt;=5.0,5.0,IF(J20&lt;=6.0,6.0,IF(J20&lt;=7.1,7.1,"two units")))))))</f>
       </c>
       <c r="L20" s="6">
-        <f>IF(J20="","",IF(J20&lt;=2.0,1650,IF(J20&lt;=2.5,1650,IF(J20&lt;=3.5,1995,IF(J20&lt;=5.0,2280,IF(J20&lt;=6.0,2650,IF(J20&lt;=7.1,2950,"")))))))</f>
+        <f>IF(J20="","",IF(J20&lt;=2.0,1650,IF(J20&lt;=2.5,1650,IF(J20&lt;=3.5,1850,IF(J20&lt;=5.0,2150,IF(J20&lt;=6.0,2450,IF(J20&lt;=7.1,2750,"")))))))</f>
       </c>
     </row>
     <row r="21">
@@ -520,7 +520,7 @@
         <f>IF(J21="","",IF(J21&lt;=2.0,2.0,IF(J21&lt;=2.5,2.5,IF(J21&lt;=3.5,3.5,IF(J21&lt;=5.0,5.0,IF(J21&lt;=6.0,6.0,IF(J21&lt;=7.1,7.1,"two units")))))))</f>
       </c>
       <c r="L21" s="6">
-        <f>IF(J21="","",IF(J21&lt;=2.0,1650,IF(J21&lt;=2.5,1650,IF(J21&lt;=3.5,1995,IF(J21&lt;=5.0,2280,IF(J21&lt;=6.0,2650,IF(J21&lt;=7.1,2950,"")))))))</f>
+        <f>IF(J21="","",IF(J21&lt;=2.0,1650,IF(J21&lt;=2.5,1650,IF(J21&lt;=3.5,1850,IF(J21&lt;=5.0,2150,IF(J21&lt;=6.0,2450,IF(J21&lt;=7.1,2750,"")))))))</f>
       </c>
     </row>
     <row r="22">
@@ -542,7 +542,7 @@
         <f>IF(J22="","",IF(J22&lt;=2.0,2.0,IF(J22&lt;=2.5,2.5,IF(J22&lt;=3.5,3.5,IF(J22&lt;=5.0,5.0,IF(J22&lt;=6.0,6.0,IF(J22&lt;=7.1,7.1,"two units")))))))</f>
       </c>
       <c r="L22" s="6">
-        <f>IF(J22="","",IF(J22&lt;=2.0,1650,IF(J22&lt;=2.5,1650,IF(J22&lt;=3.5,1995,IF(J22&lt;=5.0,2280,IF(J22&lt;=6.0,2650,IF(J22&lt;=7.1,2950,"")))))))</f>
+        <f>IF(J22="","",IF(J22&lt;=2.0,1650,IF(J22&lt;=2.5,1650,IF(J22&lt;=3.5,1850,IF(J22&lt;=5.0,2150,IF(J22&lt;=6.0,2450,IF(J22&lt;=7.1,2750,"")))))))</f>
       </c>
     </row>
     <row r="23">
@@ -564,7 +564,7 @@
         <f>IF(J23="","",IF(J23&lt;=2.0,2.0,IF(J23&lt;=2.5,2.5,IF(J23&lt;=3.5,3.5,IF(J23&lt;=5.0,5.0,IF(J23&lt;=6.0,6.0,IF(J23&lt;=7.1,7.1,"two units")))))))</f>
       </c>
       <c r="L23" s="6">
-        <f>IF(J23="","",IF(J23&lt;=2.0,1650,IF(J23&lt;=2.5,1650,IF(J23&lt;=3.5,1995,IF(J23&lt;=5.0,2280,IF(J23&lt;=6.0,2650,IF(J23&lt;=7.1,2950,"")))))))</f>
+        <f>IF(J23="","",IF(J23&lt;=2.0,1650,IF(J23&lt;=2.5,1650,IF(J23&lt;=3.5,1850,IF(J23&lt;=5.0,2150,IF(J23&lt;=6.0,2450,IF(J23&lt;=7.1,2750,"")))))))</f>
       </c>
     </row>
     <row r="24">
@@ -586,7 +586,7 @@
         <f>IF(J24="","",IF(J24&lt;=2.0,2.0,IF(J24&lt;=2.5,2.5,IF(J24&lt;=3.5,3.5,IF(J24&lt;=5.0,5.0,IF(J24&lt;=6.0,6.0,IF(J24&lt;=7.1,7.1,"two units")))))))</f>
       </c>
       <c r="L24" s="6">
-        <f>IF(J24="","",IF(J24&lt;=2.0,1650,IF(J24&lt;=2.5,1650,IF(J24&lt;=3.5,1995,IF(J24&lt;=5.0,2280,IF(J24&lt;=6.0,2650,IF(J24&lt;=7.1,2950,"")))))))</f>
+        <f>IF(J24="","",IF(J24&lt;=2.0,1650,IF(J24&lt;=2.5,1650,IF(J24&lt;=3.5,1850,IF(J24&lt;=5.0,2150,IF(J24&lt;=6.0,2450,IF(J24&lt;=7.1,2750,"")))))))</f>
       </c>
     </row>
     <row r="25">
@@ -608,7 +608,7 @@
         <f>IF(J25="","",IF(J25&lt;=2.0,2.0,IF(J25&lt;=2.5,2.5,IF(J25&lt;=3.5,3.5,IF(J25&lt;=5.0,5.0,IF(J25&lt;=6.0,6.0,IF(J25&lt;=7.1,7.1,"two units")))))))</f>
       </c>
       <c r="L25" s="6">
-        <f>IF(J25="","",IF(J25&lt;=2.0,1650,IF(J25&lt;=2.5,1650,IF(J25&lt;=3.5,1995,IF(J25&lt;=5.0,2280,IF(J25&lt;=6.0,2650,IF(J25&lt;=7.1,2950,"")))))))</f>
+        <f>IF(J25="","",IF(J25&lt;=2.0,1650,IF(J25&lt;=2.5,1650,IF(J25&lt;=3.5,1850,IF(J25&lt;=5.0,2150,IF(J25&lt;=6.0,2450,IF(J25&lt;=7.1,2750,"")))))))</f>
       </c>
     </row>
     <row r="26">
@@ -630,7 +630,7 @@
         <f>IF(J26="","",IF(J26&lt;=2.0,2.0,IF(J26&lt;=2.5,2.5,IF(J26&lt;=3.5,3.5,IF(J26&lt;=5.0,5.0,IF(J26&lt;=6.0,6.0,IF(J26&lt;=7.1,7.1,"two units")))))))</f>
       </c>
       <c r="L26" s="6">
-        <f>IF(J26="","",IF(J26&lt;=2.0,1650,IF(J26&lt;=2.5,1650,IF(J26&lt;=3.5,1995,IF(J26&lt;=5.0,2280,IF(J26&lt;=6.0,2650,IF(J26&lt;=7.1,2950,"")))))))</f>
+        <f>IF(J26="","",IF(J26&lt;=2.0,1650,IF(J26&lt;=2.5,1650,IF(J26&lt;=3.5,1850,IF(J26&lt;=5.0,2150,IF(J26&lt;=6.0,2450,IF(J26&lt;=7.1,2750,"")))))))</f>
       </c>
     </row>
     <row r="27">
@@ -652,7 +652,7 @@
         <f>IF(J27="","",IF(J27&lt;=2.0,2.0,IF(J27&lt;=2.5,2.5,IF(J27&lt;=3.5,3.5,IF(J27&lt;=5.0,5.0,IF(J27&lt;=6.0,6.0,IF(J27&lt;=7.1,7.1,"two units")))))))</f>
       </c>
       <c r="L27" s="6">
-        <f>IF(J27="","",IF(J27&lt;=2.0,1650,IF(J27&lt;=2.5,1650,IF(J27&lt;=3.5,1995,IF(J27&lt;=5.0,2280,IF(J27&lt;=6.0,2650,IF(J27&lt;=7.1,2950,"")))))))</f>
+        <f>IF(J27="","",IF(J27&lt;=2.0,1650,IF(J27&lt;=2.5,1650,IF(J27&lt;=3.5,1850,IF(J27&lt;=5.0,2150,IF(J27&lt;=6.0,2450,IF(J27&lt;=7.1,2750,"")))))))</f>
       </c>
     </row>
     <row r="28">
@@ -674,7 +674,7 @@
         <f>IF(J28="","",IF(J28&lt;=2.0,2.0,IF(J28&lt;=2.5,2.5,IF(J28&lt;=3.5,3.5,IF(J28&lt;=5.0,5.0,IF(J28&lt;=6.0,6.0,IF(J28&lt;=7.1,7.1,"two units")))))))</f>
       </c>
       <c r="L28" s="6">
-        <f>IF(J28="","",IF(J28&lt;=2.0,1650,IF(J28&lt;=2.5,1650,IF(J28&lt;=3.5,1995,IF(J28&lt;=5.0,2280,IF(J28&lt;=6.0,2650,IF(J28&lt;=7.1,2950,"")))))))</f>
+        <f>IF(J28="","",IF(J28&lt;=2.0,1650,IF(J28&lt;=2.5,1650,IF(J28&lt;=3.5,1850,IF(J28&lt;=5.0,2150,IF(J28&lt;=6.0,2450,IF(J28&lt;=7.1,2750,"")))))))</f>
       </c>
     </row>
     <row r="29">
@@ -696,7 +696,7 @@
         <f>IF(J29="","",IF(J29&lt;=2.0,2.0,IF(J29&lt;=2.5,2.5,IF(J29&lt;=3.5,3.5,IF(J29&lt;=5.0,5.0,IF(J29&lt;=6.0,6.0,IF(J29&lt;=7.1,7.1,"two units")))))))</f>
       </c>
       <c r="L29" s="6">
-        <f>IF(J29="","",IF(J29&lt;=2.0,1650,IF(J29&lt;=2.5,1650,IF(J29&lt;=3.5,1995,IF(J29&lt;=5.0,2280,IF(J29&lt;=6.0,2650,IF(J29&lt;=7.1,2950,"")))))))</f>
+        <f>IF(J29="","",IF(J29&lt;=2.0,1650,IF(J29&lt;=2.5,1650,IF(J29&lt;=3.5,1850,IF(J29&lt;=5.0,2150,IF(J29&lt;=6.0,2450,IF(J29&lt;=7.1,2750,"")))))))</f>
       </c>
     </row>
     <row r="30">

</xml_diff>